<commit_message>
Refactor dashboard and filtering UI for improved usability and aesthetics. Updated styles to use 'Inter' font, enhanced layout responsiveness, and added filter toggle functionality. Adjusted CIIU filtering options and improved overall design consistency across components.
</commit_message>
<xml_diff>
--- a/librerias_con_info_google.xlsx
+++ b/librerias_con_info_google.xlsx
@@ -670,10 +670,10 @@
         </is>
       </c>
       <c r="X2" t="n">
-        <v>187200</v>
+        <v>22770</v>
       </c>
       <c r="Y2" t="n">
-        <v>2246400</v>
+        <v>273240</v>
       </c>
       <c r="Z2" t="inlineStr">
         <is>
@@ -787,10 +787,10 @@
         </is>
       </c>
       <c r="X3" t="n">
-        <v>187200</v>
+        <v>15180</v>
       </c>
       <c r="Y3" t="n">
-        <v>2246400</v>
+        <v>182160</v>
       </c>
       <c r="Z3" t="inlineStr">
         <is>
@@ -904,10 +904,10 @@
         </is>
       </c>
       <c r="X4" t="n">
-        <v>187200</v>
+        <v>15180</v>
       </c>
       <c r="Y4" t="n">
-        <v>2246400</v>
+        <v>182160</v>
       </c>
       <c r="Z4" t="inlineStr">
         <is>
@@ -1021,10 +1021,10 @@
         </is>
       </c>
       <c r="X5" t="n">
-        <v>187200</v>
+        <v>15180</v>
       </c>
       <c r="Y5" t="n">
-        <v>2246400</v>
+        <v>182160</v>
       </c>
       <c r="Z5" t="inlineStr">
         <is>
@@ -1138,10 +1138,10 @@
         </is>
       </c>
       <c r="X6" t="n">
-        <v>158400</v>
+        <v>13860</v>
       </c>
       <c r="Y6" t="n">
-        <v>1900800</v>
+        <v>166320</v>
       </c>
       <c r="Z6" t="inlineStr">
         <is>
@@ -1251,10 +1251,10 @@
         </is>
       </c>
       <c r="X7" t="n">
-        <v>117000</v>
+        <v>9108</v>
       </c>
       <c r="Y7" t="n">
-        <v>1404000</v>
+        <v>109296</v>
       </c>
       <c r="Z7" t="inlineStr">
         <is>
@@ -1263,7 +1263,7 @@
       </c>
       <c r="AA7" t="inlineStr">
         <is>
-          <t>Basado en 82 reseñas, calificación 5</t>
+          <t>Basado en 82 reseñas, calificación 5.0</t>
         </is>
       </c>
     </row>
@@ -1364,10 +1364,10 @@
         </is>
       </c>
       <c r="X8" t="n">
-        <v>105600</v>
+        <v>13860</v>
       </c>
       <c r="Y8" t="n">
-        <v>1267200</v>
+        <v>166320</v>
       </c>
       <c r="Z8" t="inlineStr">
         <is>
@@ -1477,10 +1477,10 @@
         </is>
       </c>
       <c r="X9" t="n">
-        <v>105600</v>
+        <v>13860</v>
       </c>
       <c r="Y9" t="n">
-        <v>1267200</v>
+        <v>166320</v>
       </c>
       <c r="Z9" t="inlineStr">
         <is>
@@ -1590,10 +1590,10 @@
         </is>
       </c>
       <c r="X10" t="n">
-        <v>105600</v>
+        <v>13860</v>
       </c>
       <c r="Y10" t="n">
-        <v>1267200</v>
+        <v>166320</v>
       </c>
       <c r="Z10" t="inlineStr">
         <is>
@@ -1703,10 +1703,10 @@
         </is>
       </c>
       <c r="X11" t="n">
-        <v>105600</v>
+        <v>13860</v>
       </c>
       <c r="Y11" t="n">
-        <v>1267200</v>
+        <v>166320</v>
       </c>
       <c r="Z11" t="inlineStr">
         <is>
@@ -1816,10 +1816,10 @@
         </is>
       </c>
       <c r="X12" t="n">
-        <v>78000</v>
+        <v>9108</v>
       </c>
       <c r="Y12" t="n">
-        <v>936000</v>
+        <v>109296</v>
       </c>
       <c r="Z12" t="inlineStr">
         <is>
@@ -1925,10 +1925,10 @@
         </is>
       </c>
       <c r="X13" t="n">
-        <v>78000</v>
+        <v>9108</v>
       </c>
       <c r="Y13" t="n">
-        <v>936000</v>
+        <v>109296</v>
       </c>
       <c r="Z13" t="inlineStr">
         <is>
@@ -2034,10 +2034,10 @@
         </is>
       </c>
       <c r="X14" t="n">
-        <v>66000</v>
+        <v>8316</v>
       </c>
       <c r="Y14" t="n">
-        <v>792000</v>
+        <v>99792</v>
       </c>
       <c r="Z14" t="inlineStr">
         <is>
@@ -2143,10 +2143,10 @@
         </is>
       </c>
       <c r="X15" t="n">
-        <v>66000</v>
+        <v>8316</v>
       </c>
       <c r="Y15" t="n">
-        <v>792000</v>
+        <v>99792</v>
       </c>
       <c r="Z15" t="inlineStr">
         <is>
@@ -2155,7 +2155,7 @@
       </c>
       <c r="AA15" t="inlineStr">
         <is>
-          <t>Basado en 65 reseñas, calificación 4</t>
+          <t>Basado en 65 reseñas, calificación 4.0</t>
         </is>
       </c>
     </row>
@@ -2260,10 +2260,10 @@
         </is>
       </c>
       <c r="X16" t="n">
-        <v>58500</v>
+        <v>5313</v>
       </c>
       <c r="Y16" t="n">
-        <v>702000</v>
+        <v>63756</v>
       </c>
       <c r="Z16" t="inlineStr">
         <is>
@@ -2373,10 +2373,10 @@
         </is>
       </c>
       <c r="X17" t="n">
-        <v>58500</v>
+        <v>5313</v>
       </c>
       <c r="Y17" t="n">
-        <v>702000</v>
+        <v>63756</v>
       </c>
       <c r="Z17" t="inlineStr">
         <is>
@@ -2486,10 +2486,10 @@
         </is>
       </c>
       <c r="X18" t="n">
-        <v>58500</v>
+        <v>5313</v>
       </c>
       <c r="Y18" t="n">
-        <v>702000</v>
+        <v>63756</v>
       </c>
       <c r="Z18" t="inlineStr">
         <is>
@@ -2603,10 +2603,10 @@
         </is>
       </c>
       <c r="X19" t="n">
-        <v>58500</v>
+        <v>5313</v>
       </c>
       <c r="Y19" t="n">
-        <v>702000</v>
+        <v>63756</v>
       </c>
       <c r="Z19" t="inlineStr">
         <is>
@@ -2720,10 +2720,10 @@
         </is>
       </c>
       <c r="X20" t="n">
-        <v>58500</v>
+        <v>5313</v>
       </c>
       <c r="Y20" t="n">
-        <v>702000</v>
+        <v>63756</v>
       </c>
       <c r="Z20" t="inlineStr">
         <is>
@@ -2837,10 +2837,10 @@
         </is>
       </c>
       <c r="X21" t="n">
-        <v>58500</v>
+        <v>5313</v>
       </c>
       <c r="Y21" t="n">
-        <v>702000</v>
+        <v>63756</v>
       </c>
       <c r="Z21" t="inlineStr">
         <is>
@@ -2954,10 +2954,10 @@
         </is>
       </c>
       <c r="X22" t="n">
-        <v>49500</v>
+        <v>4851</v>
       </c>
       <c r="Y22" t="n">
-        <v>594000</v>
+        <v>58212</v>
       </c>
       <c r="Z22" t="inlineStr">
         <is>
@@ -3071,10 +3071,10 @@
         </is>
       </c>
       <c r="X23" t="n">
-        <v>45000</v>
+        <v>4620</v>
       </c>
       <c r="Y23" t="n">
-        <v>540000</v>
+        <v>55440</v>
       </c>
       <c r="Z23" t="inlineStr">
         <is>
@@ -3184,14 +3184,14 @@
         </is>
       </c>
       <c r="X24" t="n">
-        <v>39000</v>
+        <v>5313</v>
       </c>
       <c r="Y24" t="n">
-        <v>468000</v>
+        <v>63756</v>
       </c>
       <c r="Z24" t="inlineStr">
         <is>
-          <t>media</t>
+          <t>alta</t>
         </is>
       </c>
       <c r="AA24" t="inlineStr">
@@ -3293,14 +3293,14 @@
         </is>
       </c>
       <c r="X25" t="n">
-        <v>39000</v>
+        <v>5313</v>
       </c>
       <c r="Y25" t="n">
-        <v>468000</v>
+        <v>63756</v>
       </c>
       <c r="Z25" t="inlineStr">
         <is>
-          <t>media</t>
+          <t>alta</t>
         </is>
       </c>
       <c r="AA25" t="inlineStr">
@@ -3406,14 +3406,14 @@
         </is>
       </c>
       <c r="X26" t="n">
-        <v>30000</v>
+        <v>4620</v>
       </c>
       <c r="Y26" t="n">
-        <v>360000</v>
+        <v>55440</v>
       </c>
       <c r="Z26" t="inlineStr">
         <is>
-          <t>media</t>
+          <t>alta</t>
         </is>
       </c>
       <c r="AA26" t="inlineStr">
@@ -3519,10 +3519,10 @@
         </is>
       </c>
       <c r="X27" t="n">
-        <v>23400</v>
+        <v>2277</v>
       </c>
       <c r="Y27" t="n">
-        <v>280800</v>
+        <v>27324</v>
       </c>
       <c r="Z27" t="inlineStr">
         <is>
@@ -3531,7 +3531,7 @@
       </c>
       <c r="AA27" t="inlineStr">
         <is>
-          <t>Basado en 4 reseñas, calificación 5</t>
+          <t>Basado en 4 reseñas, calificación 5.0</t>
         </is>
       </c>
     </row>
@@ -3632,19 +3632,19 @@
         </is>
       </c>
       <c r="X28" t="n">
-        <v>15600</v>
+        <v>2277</v>
       </c>
       <c r="Y28" t="n">
-        <v>187200</v>
+        <v>27324</v>
       </c>
       <c r="Z28" t="inlineStr">
         <is>
-          <t>baja</t>
+          <t>alta</t>
         </is>
       </c>
       <c r="AA28" t="inlineStr">
         <is>
-          <t>Basado en 5 reseñas, calificación 5</t>
+          <t>Basado en 5 reseñas, calificación 5.0</t>
         </is>
       </c>
     </row>
@@ -3741,14 +3741,14 @@
         </is>
       </c>
       <c r="X29" t="n">
-        <v>15600</v>
+        <v>2277</v>
       </c>
       <c r="Y29" t="n">
-        <v>187200</v>
+        <v>27324</v>
       </c>
       <c r="Z29" t="inlineStr">
         <is>
-          <t>baja</t>
+          <t>alta</t>
         </is>
       </c>
       <c r="AA29" t="inlineStr">
@@ -3850,14 +3850,14 @@
         </is>
       </c>
       <c r="X30" t="n">
-        <v>15600</v>
+        <v>2277</v>
       </c>
       <c r="Y30" t="n">
-        <v>187200</v>
+        <v>27324</v>
       </c>
       <c r="Z30" t="inlineStr">
         <is>
-          <t>baja</t>
+          <t>alta</t>
         </is>
       </c>
       <c r="AA30" t="inlineStr">
@@ -3963,14 +3963,14 @@
         </is>
       </c>
       <c r="X31" t="n">
-        <v>15600</v>
+        <v>2277</v>
       </c>
       <c r="Y31" t="n">
-        <v>187200</v>
+        <v>27324</v>
       </c>
       <c r="Z31" t="inlineStr">
         <is>
-          <t>baja</t>
+          <t>alta</t>
         </is>
       </c>
       <c r="AA31" t="inlineStr">
@@ -4072,14 +4072,14 @@
         </is>
       </c>
       <c r="X32" t="n">
-        <v>15600</v>
+        <v>2277</v>
       </c>
       <c r="Y32" t="n">
-        <v>187200</v>
+        <v>27324</v>
       </c>
       <c r="Z32" t="inlineStr">
         <is>
-          <t>baja</t>
+          <t>alta</t>
         </is>
       </c>
       <c r="AA32" t="inlineStr">
@@ -4181,14 +4181,14 @@
         </is>
       </c>
       <c r="X33" t="n">
-        <v>15600</v>
+        <v>2277</v>
       </c>
       <c r="Y33" t="n">
-        <v>187200</v>
+        <v>27324</v>
       </c>
       <c r="Z33" t="inlineStr">
         <is>
-          <t>baja</t>
+          <t>alta</t>
         </is>
       </c>
       <c r="AA33" t="inlineStr">
@@ -4294,14 +4294,14 @@
         </is>
       </c>
       <c r="X34" t="n">
-        <v>15600</v>
+        <v>2277</v>
       </c>
       <c r="Y34" t="n">
-        <v>187200</v>
+        <v>27324</v>
       </c>
       <c r="Z34" t="inlineStr">
         <is>
-          <t>baja</t>
+          <t>alta</t>
         </is>
       </c>
       <c r="AA34" t="inlineStr">
@@ -4407,19 +4407,19 @@
         </is>
       </c>
       <c r="X35" t="n">
-        <v>15600</v>
+        <v>2277</v>
       </c>
       <c r="Y35" t="n">
-        <v>187200</v>
+        <v>27324</v>
       </c>
       <c r="Z35" t="inlineStr">
         <is>
-          <t>baja</t>
+          <t>alta</t>
         </is>
       </c>
       <c r="AA35" t="inlineStr">
         <is>
-          <t>Basado en 5 reseñas, calificación 5</t>
+          <t>Basado en 5 reseñas, calificación 5.0</t>
         </is>
       </c>
     </row>
@@ -4520,19 +4520,19 @@
         </is>
       </c>
       <c r="X36" t="n">
-        <v>15600</v>
+        <v>2277</v>
       </c>
       <c r="Y36" t="n">
-        <v>187200</v>
+        <v>27324</v>
       </c>
       <c r="Z36" t="inlineStr">
         <is>
-          <t>baja</t>
+          <t>alta</t>
         </is>
       </c>
       <c r="AA36" t="inlineStr">
         <is>
-          <t>Basado en 3 reseñas, calificación 5</t>
+          <t>Basado en 3 reseñas, calificación 5.0</t>
         </is>
       </c>
     </row>
@@ -4633,19 +4633,19 @@
         </is>
       </c>
       <c r="X37" t="n">
-        <v>15600</v>
+        <v>2277</v>
       </c>
       <c r="Y37" t="n">
-        <v>187200</v>
+        <v>27324</v>
       </c>
       <c r="Z37" t="inlineStr">
         <is>
-          <t>baja</t>
+          <t>alta</t>
         </is>
       </c>
       <c r="AA37" t="inlineStr">
         <is>
-          <t>Basado en 1 reseñas, calificación 5</t>
+          <t>Basado en 1 reseñas, calificación 5.0</t>
         </is>
       </c>
     </row>
@@ -4742,19 +4742,19 @@
         </is>
       </c>
       <c r="X38" t="n">
-        <v>15600</v>
+        <v>2277</v>
       </c>
       <c r="Y38" t="n">
-        <v>187200</v>
+        <v>27324</v>
       </c>
       <c r="Z38" t="inlineStr">
         <is>
-          <t>baja</t>
+          <t>alta</t>
         </is>
       </c>
       <c r="AA38" t="inlineStr">
         <is>
-          <t>Basado en 2 reseñas, calificación 5</t>
+          <t>Basado en 2 reseñas, calificación 5.0</t>
         </is>
       </c>
     </row>
@@ -4855,14 +4855,14 @@
         </is>
       </c>
       <c r="X39" t="n">
-        <v>15600</v>
+        <v>2277</v>
       </c>
       <c r="Y39" t="n">
-        <v>187200</v>
+        <v>27324</v>
       </c>
       <c r="Z39" t="inlineStr">
         <is>
-          <t>baja</t>
+          <t>alta</t>
         </is>
       </c>
       <c r="AA39" t="inlineStr">
@@ -4968,14 +4968,14 @@
         </is>
       </c>
       <c r="X40" t="n">
-        <v>15600</v>
+        <v>2277</v>
       </c>
       <c r="Y40" t="n">
-        <v>187200</v>
+        <v>27324</v>
       </c>
       <c r="Z40" t="inlineStr">
         <is>
-          <t>baja</t>
+          <t>alta</t>
         </is>
       </c>
       <c r="AA40" t="inlineStr">
@@ -5077,14 +5077,14 @@
         </is>
       </c>
       <c r="X41" t="n">
-        <v>15600</v>
+        <v>2277</v>
       </c>
       <c r="Y41" t="n">
-        <v>187200</v>
+        <v>27324</v>
       </c>
       <c r="Z41" t="inlineStr">
         <is>
-          <t>baja</t>
+          <t>alta</t>
         </is>
       </c>
       <c r="AA41" t="inlineStr">
@@ -5190,14 +5190,14 @@
         </is>
       </c>
       <c r="X42" t="n">
-        <v>15600</v>
+        <v>2277</v>
       </c>
       <c r="Y42" t="n">
-        <v>187200</v>
+        <v>27324</v>
       </c>
       <c r="Z42" t="inlineStr">
         <is>
-          <t>baja</t>
+          <t>alta</t>
         </is>
       </c>
       <c r="AA42" t="inlineStr">
@@ -5299,14 +5299,14 @@
         </is>
       </c>
       <c r="X43" t="n">
-        <v>15600</v>
+        <v>2277</v>
       </c>
       <c r="Y43" t="n">
-        <v>187200</v>
+        <v>27324</v>
       </c>
       <c r="Z43" t="inlineStr">
         <is>
-          <t>baja</t>
+          <t>alta</t>
         </is>
       </c>
       <c r="AA43" t="inlineStr">
@@ -5412,14 +5412,14 @@
         </is>
       </c>
       <c r="X44" t="n">
-        <v>15600</v>
+        <v>2277</v>
       </c>
       <c r="Y44" t="n">
-        <v>187200</v>
+        <v>27324</v>
       </c>
       <c r="Z44" t="inlineStr">
         <is>
-          <t>baja</t>
+          <t>alta</t>
         </is>
       </c>
       <c r="AA44" t="inlineStr">
@@ -5525,19 +5525,19 @@
         </is>
       </c>
       <c r="X45" t="n">
-        <v>15600</v>
+        <v>2277</v>
       </c>
       <c r="Y45" t="n">
-        <v>187200</v>
+        <v>27324</v>
       </c>
       <c r="Z45" t="inlineStr">
         <is>
-          <t>baja</t>
+          <t>alta</t>
         </is>
       </c>
       <c r="AA45" t="inlineStr">
         <is>
-          <t>Basado en 1 reseñas, calificación 5</t>
+          <t>Basado en 1 reseñas, calificación 5.0</t>
         </is>
       </c>
     </row>
@@ -5638,14 +5638,14 @@
         </is>
       </c>
       <c r="X46" t="n">
-        <v>15600</v>
+        <v>2277</v>
       </c>
       <c r="Y46" t="n">
-        <v>187200</v>
+        <v>27324</v>
       </c>
       <c r="Z46" t="inlineStr">
         <is>
-          <t>baja</t>
+          <t>alta</t>
         </is>
       </c>
       <c r="AA46" t="inlineStr">
@@ -5747,14 +5747,14 @@
         </is>
       </c>
       <c r="X47" t="n">
-        <v>15600</v>
+        <v>2277</v>
       </c>
       <c r="Y47" t="n">
-        <v>187200</v>
+        <v>27324</v>
       </c>
       <c r="Z47" t="inlineStr">
         <is>
-          <t>baja</t>
+          <t>alta</t>
         </is>
       </c>
       <c r="AA47" t="inlineStr">
@@ -5860,19 +5860,19 @@
         </is>
       </c>
       <c r="X48" t="n">
-        <v>15600</v>
+        <v>2277</v>
       </c>
       <c r="Y48" t="n">
-        <v>187200</v>
+        <v>27324</v>
       </c>
       <c r="Z48" t="inlineStr">
         <is>
-          <t>baja</t>
+          <t>alta</t>
         </is>
       </c>
       <c r="AA48" t="inlineStr">
         <is>
-          <t>Basado en 1 reseñas, calificación 5</t>
+          <t>Basado en 1 reseñas, calificación 5.0</t>
         </is>
       </c>
     </row>
@@ -5973,14 +5973,14 @@
         </is>
       </c>
       <c r="X49" t="n">
-        <v>15600</v>
+        <v>2277</v>
       </c>
       <c r="Y49" t="n">
-        <v>187200</v>
+        <v>27324</v>
       </c>
       <c r="Z49" t="inlineStr">
         <is>
-          <t>baja</t>
+          <t>alta</t>
         </is>
       </c>
       <c r="AA49" t="inlineStr">
@@ -6086,14 +6086,14 @@
         </is>
       </c>
       <c r="X50" t="n">
-        <v>15600</v>
+        <v>2277</v>
       </c>
       <c r="Y50" t="n">
-        <v>187200</v>
+        <v>27324</v>
       </c>
       <c r="Z50" t="inlineStr">
         <is>
-          <t>baja</t>
+          <t>alta</t>
         </is>
       </c>
       <c r="AA50" t="inlineStr">
@@ -6199,19 +6199,19 @@
         </is>
       </c>
       <c r="X51" t="n">
-        <v>15600</v>
+        <v>2277</v>
       </c>
       <c r="Y51" t="n">
-        <v>187200</v>
+        <v>27324</v>
       </c>
       <c r="Z51" t="inlineStr">
         <is>
-          <t>baja</t>
+          <t>alta</t>
         </is>
       </c>
       <c r="AA51" t="inlineStr">
         <is>
-          <t>Basado en 5 reseñas, calificación 5</t>
+          <t>Basado en 5 reseñas, calificación 5.0</t>
         </is>
       </c>
     </row>
@@ -6308,19 +6308,19 @@
         </is>
       </c>
       <c r="X52" t="n">
-        <v>13200</v>
+        <v>2079</v>
       </c>
       <c r="Y52" t="n">
-        <v>158400</v>
+        <v>24948</v>
       </c>
       <c r="Z52" t="inlineStr">
         <is>
-          <t>baja</t>
+          <t>alta</t>
         </is>
       </c>
       <c r="AA52" t="inlineStr">
         <is>
-          <t>Basado en 4 reseñas, calificación 4</t>
+          <t>Basado en 4 reseñas, calificación 4.0</t>
         </is>
       </c>
     </row>
@@ -6421,14 +6421,14 @@
         </is>
       </c>
       <c r="X53" t="n">
-        <v>13200</v>
+        <v>2079</v>
       </c>
       <c r="Y53" t="n">
-        <v>158400</v>
+        <v>24948</v>
       </c>
       <c r="Z53" t="inlineStr">
         <is>
-          <t>baja</t>
+          <t>alta</t>
         </is>
       </c>
       <c r="AA53" t="inlineStr">
@@ -6530,14 +6530,14 @@
         </is>
       </c>
       <c r="X54" t="n">
-        <v>13200</v>
+        <v>2079</v>
       </c>
       <c r="Y54" t="n">
-        <v>158400</v>
+        <v>24948</v>
       </c>
       <c r="Z54" t="inlineStr">
         <is>
-          <t>baja</t>
+          <t>alta</t>
         </is>
       </c>
       <c r="AA54" t="inlineStr">
@@ -6643,14 +6643,14 @@
         </is>
       </c>
       <c r="X55" t="n">
-        <v>12000</v>
+        <v>1980</v>
       </c>
       <c r="Y55" t="n">
-        <v>144000</v>
+        <v>23760</v>
       </c>
       <c r="Z55" t="inlineStr">
         <is>
-          <t>baja</t>
+          <t>alta</t>
         </is>
       </c>
       <c r="AA55" t="inlineStr">
@@ -6752,19 +6752,19 @@
         </is>
       </c>
       <c r="X56" t="n">
-        <v>4800</v>
+        <v>950.4</v>
       </c>
       <c r="Y56" t="n">
-        <v>57600</v>
+        <v>11404.8</v>
       </c>
       <c r="Z56" t="inlineStr">
         <is>
-          <t>baja</t>
+          <t>alta</t>
         </is>
       </c>
       <c r="AA56" t="inlineStr">
         <is>
-          <t>Basado en 0 reseñas, calificación 0</t>
+          <t>Basado en 0 reseñas, calificación 0.0</t>
         </is>
       </c>
     </row>
@@ -6865,19 +6865,19 @@
         </is>
       </c>
       <c r="X57" t="n">
-        <v>4800</v>
+        <v>950.4</v>
       </c>
       <c r="Y57" t="n">
-        <v>57600</v>
+        <v>11404.8</v>
       </c>
       <c r="Z57" t="inlineStr">
         <is>
-          <t>baja</t>
+          <t>alta</t>
         </is>
       </c>
       <c r="AA57" t="inlineStr">
         <is>
-          <t>Basado en 0 reseñas, calificación 0</t>
+          <t>Basado en 0 reseñas, calificación 0.0</t>
         </is>
       </c>
     </row>
@@ -6978,19 +6978,19 @@
         </is>
       </c>
       <c r="X58" t="n">
-        <v>4800</v>
+        <v>950.4</v>
       </c>
       <c r="Y58" t="n">
-        <v>57600</v>
+        <v>11404.8</v>
       </c>
       <c r="Z58" t="inlineStr">
         <is>
-          <t>baja</t>
+          <t>alta</t>
         </is>
       </c>
       <c r="AA58" t="inlineStr">
         <is>
-          <t>Basado en 0 reseñas, calificación 0</t>
+          <t>Basado en 0 reseñas, calificación 0.0</t>
         </is>
       </c>
     </row>
@@ -7087,19 +7087,19 @@
         </is>
       </c>
       <c r="X59" t="n">
-        <v>4800</v>
+        <v>950.4</v>
       </c>
       <c r="Y59" t="n">
-        <v>57600</v>
+        <v>11404.8</v>
       </c>
       <c r="Z59" t="inlineStr">
         <is>
-          <t>baja</t>
+          <t>alta</t>
         </is>
       </c>
       <c r="AA59" t="inlineStr">
         <is>
-          <t>Basado en 0 reseñas, calificación 0</t>
+          <t>Basado en 0 reseñas, calificación 0.0</t>
         </is>
       </c>
     </row>

</xml_diff>